<commit_message>
sync all recent changes
</commit_message>
<xml_diff>
--- a/trash/17개_광역의_인구_수_변화_최근_3개월_20260226.xlsx
+++ b/trash/17개_광역의_인구_수_변화_최근_3개월_20260226.xlsx
@@ -510,8 +510,10 @@
           <t>행정구역(시군구)별</t>
         </is>
       </c>
-      <c r="B2" t="n">
-        <v>9305678</v>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>9305678</t>
+        </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -595,8 +597,10 @@
           <t>행정구역(시군구)별</t>
         </is>
       </c>
-      <c r="B3" t="n">
-        <v>9299548</v>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>9299548</t>
+        </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -680,8 +684,10 @@
           <t>행정구역(시군구)별</t>
         </is>
       </c>
-      <c r="B4" t="n">
-        <v>9299701</v>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>9299701</t>
+        </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -765,8 +771,10 @@
           <t>행정구역(시군구)별</t>
         </is>
       </c>
-      <c r="B5" t="n">
-        <v>3243759</v>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>3243759</t>
+        </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -850,8 +858,10 @@
           <t>행정구역(시군구)별</t>
         </is>
       </c>
-      <c r="B6" t="n">
-        <v>3241600</v>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>3241600</t>
+        </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -935,8 +945,10 @@
           <t>행정구역(시군구)별</t>
         </is>
       </c>
-      <c r="B7" t="n">
-        <v>3239711</v>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>3239711</t>
+        </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1020,8 +1032,10 @@
           <t>행정구역(시군구)별</t>
         </is>
       </c>
-      <c r="B8" t="n">
-        <v>2354398</v>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2354398</t>
+        </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -1105,8 +1119,10 @@
           <t>행정구역(시군구)별</t>
         </is>
       </c>
-      <c r="B9" t="n">
-        <v>2353032</v>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2353032</t>
+        </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1190,8 +1206,10 @@
           <t>행정구역(시군구)별</t>
         </is>
       </c>
-      <c r="B10" t="n">
-        <v>2352249</v>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2352249</t>
+        </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1275,8 +1293,10 @@
           <t>행정구역(시군구)별</t>
         </is>
       </c>
-      <c r="B11" t="n">
-        <v>3050547</v>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>3050547</t>
+        </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1360,8 +1380,10 @@
           <t>행정구역(시군구)별</t>
         </is>
       </c>
-      <c r="B12" t="n">
-        <v>3051961</v>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>3051961</t>
+        </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1445,8 +1467,10 @@
           <t>행정구역(시군구)별</t>
         </is>
       </c>
-      <c r="B13" t="n">
-        <v>3053308</v>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>3053308</t>
+        </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -1530,8 +1554,10 @@
           <t>행정구역(시군구)별</t>
         </is>
       </c>
-      <c r="B14" t="n">
-        <v>1394301</v>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>1394301</t>
+        </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -1615,8 +1641,10 @@
           <t>행정구역(시군구)별</t>
         </is>
       </c>
-      <c r="B15" t="n">
-        <v>1392013</v>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>1392013</t>
+        </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -1700,8 +1728,10 @@
           <t>행정구역(시군구)별</t>
         </is>
       </c>
-      <c r="B16" t="n">
-        <v>1390658</v>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>1390658</t>
+        </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -1785,8 +1815,10 @@
           <t>행정구역(시군구)별</t>
         </is>
       </c>
-      <c r="B17" t="n">
-        <v>1441886</v>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>1441886</t>
+        </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -1870,8 +1902,10 @@
           <t>행정구역(시군구)별</t>
         </is>
       </c>
-      <c r="B18" t="n">
-        <v>1440729</v>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>1440729</t>
+        </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -1955,8 +1989,10 @@
           <t>행정구역(시군구)별</t>
         </is>
       </c>
-      <c r="B19" t="n">
-        <v>1440550</v>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>1440550</t>
+        </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -2040,8 +2076,10 @@
           <t>행정구역(시군구)별</t>
         </is>
       </c>
-      <c r="B20" t="n">
-        <v>1092573</v>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>1092573</t>
+        </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -2125,8 +2163,10 @@
           <t>행정구역(시군구)별</t>
         </is>
       </c>
-      <c r="B21" t="n">
-        <v>1091948</v>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>1091948</t>
+        </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -2210,8 +2250,10 @@
           <t>행정구역(시군구)별</t>
         </is>
       </c>
-      <c r="B22" t="n">
-        <v>1091281</v>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>1091281</t>
+        </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -2295,8 +2337,10 @@
           <t>행정구역(시군구)별</t>
         </is>
       </c>
-      <c r="B23" t="n">
-        <v>392495</v>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>392495</t>
+        </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -2380,8 +2424,10 @@
           <t>행정구역(시군구)별</t>
         </is>
       </c>
-      <c r="B24" t="n">
-        <v>391965</v>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>391965</t>
+        </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -2465,8 +2511,10 @@
           <t>행정구역(시군구)별</t>
         </is>
       </c>
-      <c r="B25" t="n">
-        <v>391477</v>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>391477</t>
+        </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -2550,8 +2598,10 @@
           <t>행정구역(시군구)별</t>
         </is>
       </c>
-      <c r="B26" t="n">
-        <v>13725710</v>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>13725710</t>
+        </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -2635,8 +2685,10 @@
           <t>행정구역(시군구)별</t>
         </is>
       </c>
-      <c r="B27" t="n">
-        <v>13730135</v>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>13730135</t>
+        </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -2720,8 +2772,10 @@
           <t>행정구역(시군구)별</t>
         </is>
       </c>
-      <c r="B28" t="n">
-        <v>13736642</v>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>13736642</t>
+        </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -2805,8 +2859,10 @@
           <t>행정구역(시군구)별</t>
         </is>
       </c>
-      <c r="B29" t="n">
-        <v>1593151</v>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>1593151</t>
+        </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -2890,8 +2946,10 @@
           <t>행정구역(시군구)별</t>
         </is>
       </c>
-      <c r="B30" t="n">
-        <v>1596502</v>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>1596502</t>
+        </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -2975,8 +3033,10 @@
           <t>행정구역(시군구)별</t>
         </is>
       </c>
-      <c r="B31" t="n">
-        <v>1596749</v>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>1596749</t>
+        </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -3060,8 +3120,10 @@
           <t>행정구역(시군구)별</t>
         </is>
       </c>
-      <c r="B32" t="n">
-        <v>2136966</v>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2136966</t>
+        </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -3145,8 +3207,10 @@
           <t>행정구역(시군구)별</t>
         </is>
       </c>
-      <c r="B33" t="n">
-        <v>2136753</v>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2136753</t>
+        </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -3230,8 +3294,10 @@
           <t>행정구역(시군구)별</t>
         </is>
       </c>
-      <c r="B34" t="n">
-        <v>2136204</v>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2136204</t>
+        </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -3315,8 +3381,10 @@
           <t>행정구역(시군구)별</t>
         </is>
       </c>
-      <c r="B35" t="n">
-        <v>1779242</v>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>1779242</t>
+        </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -3400,8 +3468,10 @@
           <t>행정구역(시군구)별</t>
         </is>
       </c>
-      <c r="B36" t="n">
-        <v>1779135</v>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>1779135</t>
+        </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -3485,8 +3555,10 @@
           <t>행정구역(시군구)별</t>
         </is>
       </c>
-      <c r="B37" t="n">
-        <v>1778171</v>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>1778171</t>
+        </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -3570,8 +3642,10 @@
           <t>행정구역(시군구)별</t>
         </is>
       </c>
-      <c r="B38" t="n">
-        <v>2509131</v>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>2509131</t>
+        </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -3655,8 +3729,10 @@
           <t>행정구역(시군구)별</t>
         </is>
       </c>
-      <c r="B39" t="n">
-        <v>2506526</v>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>2506526</t>
+        </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -3740,8 +3816,10 @@
           <t>행정구역(시군구)별</t>
         </is>
       </c>
-      <c r="B40" t="n">
-        <v>2503544</v>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>2503544</t>
+        </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -3825,8 +3903,10 @@
           <t>행정구역(시군구)별</t>
         </is>
       </c>
-      <c r="B41" t="n">
-        <v>3208860</v>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>3208860</t>
+        </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -3910,8 +3990,10 @@
           <t>행정구역(시군구)별</t>
         </is>
       </c>
-      <c r="B42" t="n">
-        <v>3207383</v>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>3207383</t>
+        </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -3995,8 +4077,10 @@
           <t>행정구역(시군구)별</t>
         </is>
       </c>
-      <c r="B43" t="n">
-        <v>3205787</v>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>3205787</t>
+        </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -4080,8 +4164,10 @@
           <t>행정구역(시군구)별</t>
         </is>
       </c>
-      <c r="B44" t="n">
-        <v>664922</v>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>664922</t>
+        </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -4165,8 +4251,10 @@
           <t>행정구역(시군구)별</t>
         </is>
       </c>
-      <c r="B45" t="n">
-        <v>664792</v>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>664792</t>
+        </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -4250,8 +4338,10 @@
           <t>행정구역(시군구)별</t>
         </is>
       </c>
-      <c r="B46" t="n">
-        <v>663995</v>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>663995</t>
+        </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -4335,8 +4425,10 @@
           <t>행정구역(시군구)별</t>
         </is>
       </c>
-      <c r="B47" t="n">
-        <v>1508951</v>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>1508951</t>
+        </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -4420,8 +4512,10 @@
           <t>행정구역(시군구)별</t>
         </is>
       </c>
-      <c r="B48" t="n">
-        <v>1508500</v>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>1508500</t>
+        </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -4505,8 +4599,10 @@
           <t>행정구역(시군구)별</t>
         </is>
       </c>
-      <c r="B49" t="n">
-        <v>1507634</v>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>1507634</t>
+        </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -4590,8 +4686,10 @@
           <t>행정구역(시군구)별</t>
         </is>
       </c>
-      <c r="B50" t="n">
-        <v>1725960</v>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>1725960</t>
+        </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
@@ -4675,8 +4773,10 @@
           <t>행정구역(시군구)별</t>
         </is>
       </c>
-      <c r="B51" t="n">
-        <v>1724856</v>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>1724856</t>
+        </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
@@ -4760,8 +4860,10 @@
           <t>행정구역(시군구)별</t>
         </is>
       </c>
-      <c r="B52" t="n">
-        <v>1723497</v>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>1723497</t>
+        </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>

</xml_diff>